<commit_message>
[Chore] So 데이터 수정
</commit_message>
<xml_diff>
--- a/Assets/08.Excel/GameData.xlsx
+++ b/Assets/08.Excel/GameData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\My idle game\my-idle-game\Assets\08.Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0B1B321-3C3D-42B3-90C4-7AAAF4753ABD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DCC0C5A-6F50-4387-808C-E98F58D57D1F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8856" activeTab="2" xr2:uid="{698F8AFA-8894-42B5-A618-49D138110CB8}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8856" activeTab="1" xr2:uid="{698F8AFA-8894-42B5-A618-49D138110CB8}"/>
   </bookViews>
   <sheets>
     <sheet name="ItemSheet" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="74">
   <si>
     <t>Id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -312,96 +312,7 @@
   </si>
   <si>
     <t>Assets/00.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/01.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/02.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/03.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/04.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/05.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/06.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/07.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/08.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/09.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/10.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/11.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/12.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/13.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/14.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/15.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/16.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/17.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/18.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/19.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/20.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/21.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/22.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/23.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/24.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/25.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/26.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/27.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/28.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/29.Externals/Myaddressable/G_coin.png[G_coin]</t>
-  </si>
-  <si>
-    <t>Assets/30.Externals/Myaddressable/G_coin.png[G_coin]</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -809,7 +720,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1002,6 +913,18 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1024,15 +947,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2058,8 +1972,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"002"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201002001</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>74</v>
+      <c r="B3" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C3" s="62">
         <v>10000</v>
@@ -2070,8 +1984,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"003"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201003001</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>75</v>
+      <c r="B4" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C4" s="62">
         <v>15000</v>
@@ -2082,8 +1996,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"004"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201004001</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>76</v>
+      <c r="B5" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C5" s="62">
         <v>20000</v>
@@ -2094,8 +2008,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"005"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201005001</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>77</v>
+      <c r="B6" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C6" s="62">
         <v>5000</v>
@@ -2106,8 +2020,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"006"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201006001</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>78</v>
+      <c r="B7" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C7" s="62">
         <v>8000</v>
@@ -2118,8 +2032,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"007"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201007001</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>79</v>
+      <c r="B8" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C8" s="62">
         <v>9000</v>
@@ -2130,8 +2044,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"008"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201008001</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>80</v>
+      <c r="B9" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C9" s="62">
         <v>10000</v>
@@ -2142,8 +2056,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"009"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201009001</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>81</v>
+      <c r="B10" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C10" s="62">
         <v>10000</v>
@@ -2154,8 +2068,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"010"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201010001</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>82</v>
+      <c r="B11" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C11" s="62">
         <v>15000</v>
@@ -2166,8 +2080,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"011"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201011001</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>83</v>
+      <c r="B12" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C12" s="62">
         <v>20000</v>
@@ -2178,8 +2092,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"012"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201012001</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>84</v>
+      <c r="B13" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C13" s="62">
         <v>5000</v>
@@ -2190,8 +2104,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"013"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201013001</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>85</v>
+      <c r="B14" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C14" s="62">
         <v>8000</v>
@@ -2202,8 +2116,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"014"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201014001</v>
       </c>
-      <c r="B15" s="1" t="s">
-        <v>86</v>
+      <c r="B15" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C15" s="62">
         <v>9000</v>
@@ -2214,8 +2128,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"015"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201015001</v>
       </c>
-      <c r="B16" s="1" t="s">
-        <v>87</v>
+      <c r="B16" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C16" s="62">
         <v>10000</v>
@@ -2226,8 +2140,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"016"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201016001</v>
       </c>
-      <c r="B17" s="1" t="s">
-        <v>88</v>
+      <c r="B17" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C17" s="62">
         <v>10000</v>
@@ -2238,8 +2152,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"017"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201017001</v>
       </c>
-      <c r="B18" s="1" t="s">
-        <v>89</v>
+      <c r="B18" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C18" s="62">
         <v>15000</v>
@@ -2250,8 +2164,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"018"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201018001</v>
       </c>
-      <c r="B19" s="1" t="s">
-        <v>90</v>
+      <c r="B19" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C19" s="62">
         <v>20000</v>
@@ -2262,8 +2176,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"019"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201019001</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>91</v>
+      <c r="B20" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C20" s="62">
         <v>5000</v>
@@ -2274,8 +2188,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"020"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201020001</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>92</v>
+      <c r="B21" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C21" s="62">
         <v>8000</v>
@@ -2286,8 +2200,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"021"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201021001</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>93</v>
+      <c r="B22" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C22" s="62">
         <v>9000</v>
@@ -2298,8 +2212,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"022"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201022001</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>94</v>
+      <c r="B23" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C23" s="62">
         <v>10000</v>
@@ -2310,8 +2224,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"023"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201023001</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>95</v>
+      <c r="B24" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C24" s="62">
         <v>10000</v>
@@ -2322,8 +2236,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"024"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201024001</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>96</v>
+      <c r="B25" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C25" s="62">
         <v>15000</v>
@@ -2334,8 +2248,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"025"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201025001</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>97</v>
+      <c r="B26" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C26" s="62">
         <v>20000</v>
@@ -2346,8 +2260,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"026"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201026001</v>
       </c>
-      <c r="B27" s="1" t="s">
-        <v>98</v>
+      <c r="B27" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C27" s="62">
         <v>5000</v>
@@ -2358,8 +2272,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"027"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201027001</v>
       </c>
-      <c r="B28" s="1" t="s">
-        <v>99</v>
+      <c r="B28" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C28" s="62">
         <v>8000</v>
@@ -2370,8 +2284,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"028"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201028001</v>
       </c>
-      <c r="B29" s="1" t="s">
-        <v>100</v>
+      <c r="B29" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C29" s="62">
         <v>9000</v>
@@ -2382,8 +2296,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"029"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201029001</v>
       </c>
-      <c r="B30" s="1" t="s">
-        <v>101</v>
+      <c r="B30" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C30" s="62">
         <v>10000</v>
@@ -2394,8 +2308,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"030"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201030001</v>
       </c>
-      <c r="B31" s="1" t="s">
-        <v>102</v>
+      <c r="B31" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C31" s="62">
         <v>10000</v>
@@ -2406,8 +2320,8 @@
         <f>TEXT(규칙!$B$4,"000")&amp;"031"&amp;TEXT(규칙!$H$9,"000")</f>
         <v>201031001</v>
       </c>
-      <c r="B32" s="1" t="s">
-        <v>103</v>
+      <c r="B32" s="64" t="s">
+        <v>73</v>
       </c>
       <c r="C32" s="62">
         <v>15000</v>
@@ -2444,25 +2358,25 @@
       <c r="A2" s="58" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="66" t="s">
+      <c r="B2" s="70" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="67"/>
+      <c r="C2" s="71"/>
       <c r="D2" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="66" t="s">
+      <c r="E2" s="70" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="67"/>
+      <c r="F2" s="71"/>
       <c r="G2" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="H2" s="66" t="s">
+      <c r="H2" s="70" t="s">
         <v>18</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="K2" s="68" t="s">
+      <c r="I2" s="71"/>
+      <c r="K2" s="72" t="s">
         <v>44</v>
       </c>
       <c r="L2" s="12" t="s">
@@ -2492,7 +2406,7 @@
       <c r="I3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" s="68"/>
+      <c r="K3" s="72"/>
       <c r="L3" s="12" t="s">
         <v>24</v>
       </c>
@@ -2536,7 +2450,7 @@
       <c r="I5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K5" s="71" t="s">
+      <c r="K5" s="75" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2555,7 +2469,7 @@
       <c r="I6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="K6" s="71"/>
+      <c r="K6" s="75"/>
     </row>
     <row r="7" spans="1:13" ht="18" thickBot="1" x14ac:dyDescent="0.45"/>
     <row r="8" spans="1:13" ht="18" thickBot="1" x14ac:dyDescent="0.45">
@@ -2571,17 +2485,17 @@
       <c r="D8" s="61" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="69" t="s">
+      <c r="E8" s="73" t="s">
         <v>66</v>
       </c>
-      <c r="F8" s="70"/>
+      <c r="F8" s="74"/>
       <c r="G8" s="63" t="s">
         <v>61</v>
       </c>
-      <c r="H8" s="69" t="s">
+      <c r="H8" s="73" t="s">
         <v>63</v>
       </c>
-      <c r="I8" s="70"/>
+      <c r="I8" s="74"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A9" s="18" t="s">
@@ -2616,10 +2530,10 @@
       <c r="C10" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="64" t="s">
+      <c r="E10" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="65"/>
+      <c r="F10" s="69"/>
       <c r="H10" s="9">
         <v>2</v>
       </c>
@@ -2685,7 +2599,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A17" s="74"/>
+      <c r="A17" s="67"/>
       <c r="B17" s="6"/>
       <c r="C17" s="6"/>
     </row>
@@ -2707,11 +2621,11 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B22" s="6"/>
-      <c r="C22" s="72"/>
+      <c r="C22" s="65"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="B23" s="6"/>
-      <c r="C23" s="73"/>
+      <c r="C23" s="66"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>